<commit_message>
CI Reports [2026-06-24 18:48]: Dashboard — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/DailyBugReport_2026-06-24.xlsx
+++ b/Test Execution Report/Daily Reports/DailyBugReport_2026-06-24.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O7"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -510,9 +510,254 @@
         <v>Clean run — 6/24/2026, 6:27:53 PM</v>
       </c>
     </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>24 Jun 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>BUG-DASHBOARD-001</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="E3" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H3" t="str">
+        <v>New</v>
+      </c>
+      <c r="I3" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N3" t="str">
+        <v>reports/screenshots/TC-DASH-002-failure.png</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>24 Jun 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BUG-DASHBOARD-002</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="E4" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H4" t="str">
+        <v>New</v>
+      </c>
+      <c r="I4" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N4" t="str">
+        <v>reports/screenshots/TC-DASH-004-failure.png</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>24 Jun 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>BUG-DASHBOARD-003</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="E5" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H5" t="str">
+        <v>New</v>
+      </c>
+      <c r="I5" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N5" t="str">
+        <v>reports/screenshots/TC-DASH-005-failure.png</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>24 Jun 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BUG-DASHBOARD-004</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="E6" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H6" t="str">
+        <v>New</v>
+      </c>
+      <c r="I6" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('button:has-text("Reset")').first() Expected: visible Received: hidden Timeout:  5000ms  Ca</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N6" t="str">
+        <v>reports/screenshots/TC-DASH-007-failure.png</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>24 Jun 2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BUG-DASHBOARD-005</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="E7" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G7" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H7" t="str">
+        <v>New</v>
+      </c>
+      <c r="I7" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N7" t="str">
+        <v>reports/screenshots/TC-DASH-011-failure.png</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>